<commit_message>
Updated schedule.xlsx with new entries
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20" count="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19" count="21">
   <si>
     <t>Publish</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>/slides/01-welcome.qmd</t>
-  </si>
-  <si>
-    <t>/ae/ae-01-multivariate-relationships.qmd</t>
   </si>
   <si>
     <t>Welcome!</t>
@@ -337,13 +334,11 @@
       <c r="G2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="H2" s="6"/>
       <c r="I2" s="10"/>
       <c r="J2" s="9"/>
       <c r="K2" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L2" s="6"/>
     </row>
@@ -361,10 +356,10 @@
         <v>45903</v>
       </c>
       <c r="E3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
       </c>
       <c r="G3" s="6"/>
       <c r="H3" s="4"/>

</xml_diff>

<commit_message>
Add preparation materials and slides for MATH 2025 course
- Created new preparation document for "Preparation for the Big Picture" (prep-01.qmd).
- Updated "Preparation for Simple Linear Regression" to "Preparation for Multivariate Relationships" (prep-02.qmd).
- Added new preparation document for "Preparation for Simulation Based Inference" (prep-03-01.qmd).
- Updated "Preparation for Simulation Based Inference" content in prep-03.qmd.
- Updated schedule.xlsx with new course information.
- Created welcome slide deck for MATH 2025 (00-welcome.qmd).
- Created slide deck for "The Big Picture" (01-big-picture.qmd).
- Created slide deck for "Multivariate Relationships" (01-multivariate-relationships.qmd).
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19" count="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27" count="32">
   <si>
     <t>Publish</t>
   </si>
@@ -61,16 +61,40 @@
     <t>Welcome to MATH 2025!</t>
   </si>
   <si>
-    <t>/slides/01-welcome.qmd</t>
+    <t>/slides/00-welcome.qmd</t>
   </si>
   <si>
     <t>Welcome!</t>
   </si>
   <si>
-    <t>Multivariate Relationsihps</t>
+    <t>The Big Picture</t>
+  </si>
+  <si>
+    <t>/prepare/prep-01.qmd</t>
+  </si>
+  <si>
+    <t>/slides/01-big-picture.qmd</t>
+  </si>
+  <si>
+    <t>/ae/ae-01-getting-started.qmd</t>
+  </si>
+  <si>
+    <t>Our first AE!</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>ultivariate Relationships</t>
   </si>
   <si>
     <t>/prepare/prep-02.qmd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Simple Linear Regression </t>
+  </si>
+  <si>
+    <t>/prepare/prep-03.qmd</t>
   </si>
 </sst>
 </file>
@@ -319,7 +343,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>13</v>
@@ -347,7 +371,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>13</v>
@@ -361,20 +385,38 @@
       <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="6"/>
-      <c r="H3" s="4"/>
+      <c r="G3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
+      <c r="K3" s="9" t="s">
+        <v>21</v>
+      </c>
       <c r="L3" s="6"/>
     </row>
     <row r="4" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="9"/>
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="5">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="7">
+        <v>45908</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
       <c r="G4" s="6"/>
       <c r="H4" s="4"/>
       <c r="I4" s="9"/>
@@ -383,12 +425,24 @@
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A5" s="4"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="9"/>
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="7">
+        <v>45910</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
       <c r="G5" s="6"/>
       <c r="H5" s="4"/>
       <c r="I5" s="9"/>

</xml_diff>

<commit_message>
Updated lecture 4 and added lecutre 5
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,20 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\efriedlander\Documents\Teaching\MATH2025FA25\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{859E1DB6-5A61-4652-B23E-9D680FA80414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullPrecision="1" calcId="125725"/>
+  <calcPr calcId="125725"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="35" count="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>Publish</t>
   </si>
@@ -119,104 +131,81 @@
   </si>
   <si>
     <t>/prepare/prep-04.qmd</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Testing and Confidence Intervals</t>
+  </si>
+  <si>
+    <t>/slides/04-slr-fit-prediction.qmd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <fonts count="14">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Aptos Narrow"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Open Sans"/>
-      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
-      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Open Sans"/>
-      <charset val="0"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="0"/>
     </font>
     <font>
-      <sz val="0"/>
+      <sz val="1"/>
       <color rgb="FF334052"/>
       <name val="Inter, sans-serif"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="0"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color rgb="FF467886"/>
       <name val="Aptos Narrow"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFB0280"/>
       <name val="Open Sans"/>
-      <charset val="0"/>
     </font>
   </fonts>
   <fills count="7">
     <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="64"/>
-        <bgColor indexed="65"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor indexed="64"/>
-        <bgColor indexed="65"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -273,78 +262,356 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="38">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs>
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf numFmtId="16" fontId="6" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="18" fontId="11" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Sheet1LockedColumnStyle" xfId="20"/>
-    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="21"/>
+    <cellStyle name="Sheet1LockedColumnStyle" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L53"/>
-  <sheetFormatPr customHeight="true" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="7" max="7" width="41" customWidth="1"/>
   </cols>
@@ -511,22 +778,28 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="5"/>
+      <c r="B6" s="5">
+        <v>4</v>
+      </c>
       <c r="C6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="7">
         <v>45915</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="12" t="s">
-        <v>32</v>
-      </c>
+      <c r="E6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="9"/>
       <c r="J6" s="9"/>
       <c r="K6" s="9"/>
       <c r="L6" s="6"/>
@@ -536,19 +809,16 @@
         <v>12</v>
       </c>
       <c r="B7" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D7" s="7">
-        <v>45915</v>
+        <v>45917</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="4"/>
@@ -558,18 +828,28 @@
       <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A8" s="4"/>
+      <c r="A8" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="B8" s="5"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="4"/>
+      <c r="C8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="7">
+        <v>45919</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="F8" s="9"/>
-      <c r="G8" s="4"/>
+      <c r="G8" s="6"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="I8" s="12" t="s">
+        <v>32</v>
+      </c>
       <c r="J8" s="9"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="6"/>
     </row>
     <row r="9" spans="1:12" ht="16.5" customHeight="1">
       <c r="A9" s="4"/>
@@ -1089,7 +1369,7 @@
       <c r="K45" s="6"/>
       <c r="L45" s="9"/>
     </row>
-    <row r="46" spans="1:12" ht="16.5" customHeight="1">
+    <row r="46" spans="1:12" ht="86.25" customHeight="1">
       <c r="A46" s="4"/>
       <c r="B46" s="14"/>
       <c r="C46" s="6"/>
@@ -1103,7 +1383,7 @@
       <c r="K46" s="9"/>
       <c r="L46" s="6"/>
     </row>
-    <row r="47" spans="1:12" ht="86.25" customHeight="1">
+    <row r="47" spans="1:12" ht="16.5" customHeight="1">
       <c r="A47" s="4"/>
       <c r="B47" s="14"/>
       <c r="C47" s="6"/>
@@ -1187,7 +1467,7 @@
       <c r="K52" s="9"/>
       <c r="L52" s="9"/>
     </row>
-    <row r="53" spans="1:12" ht="16.5" customHeight="1">
+    <row r="53" spans="1:12" ht="15" customHeight="1">
       <c r="A53" s="4"/>
       <c r="B53" s="14"/>
       <c r="C53" s="6"/>
@@ -1203,7 +1483,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>
-  <extLst/>
+  <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added deepnote for AE-05
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="39" count="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="40" count="51">
   <si>
     <t>Publish</t>
   </si>
@@ -122,6 +122,9 @@
   </si>
   <si>
     <t>/prepare/prep-05.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-05-Hypothesis-Testing-a50d53f1-7c77-4add-8c8b-898d3ea049d6/notebook/ae-05-sbi-ht-82aa13654bfb4659bfce3a86d4d4c28e?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=a50d53f1-7c77-4add-8c8b-898d3ea049d6</t>
   </si>
   <si>
     <t>F</t>
@@ -137,7 +140,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -192,6 +195,12 @@
     </font>
     <font>
       <sz val="1"/>
+      <color rgb="FF334052"/>
+      <name val="Inter, sans-serif"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="0"/>
       <color rgb="FF334052"/>
       <name val="Inter, sans-serif"/>
       <charset val="0"/>
@@ -217,7 +226,7 @@
       <charset val="0"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none">
         <fgColor indexed="64"/>
@@ -254,6 +263,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -279,7 +294,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="38">
+  <cellStyleXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
@@ -324,10 +339,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="18" fontId="11" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyFill="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="18" fontId="12" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -563,7 +581,9 @@
         <v>35</v>
       </c>
       <c r="G7" s="6"/>
-      <c r="H7" s="4"/>
+      <c r="H7" s="12" t="s">
+        <v>36</v>
+      </c>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
@@ -575,19 +595,19 @@
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="7">
         <v>45919</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F8" s="9"/>
       <c r="G8" s="6"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="12" t="s">
-        <v>38</v>
+      <c r="I8" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
@@ -729,7 +749,7 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="13"/>
+      <c r="J18" s="14"/>
       <c r="K18" s="6"/>
       <c r="L18" s="9"/>
     </row>
@@ -777,7 +797,7 @@
     </row>
     <row r="22" spans="1:12" ht="16.5" customHeight="1">
       <c r="A22" s="4"/>
-      <c r="B22" s="14"/>
+      <c r="B22" s="15"/>
       <c r="C22" s="6"/>
       <c r="D22" s="7"/>
       <c r="E22" s="8"/>
@@ -791,7 +811,7 @@
     </row>
     <row r="23" spans="1:12" ht="16.5" customHeight="1">
       <c r="A23" s="4"/>
-      <c r="B23" s="14"/>
+      <c r="B23" s="15"/>
       <c r="C23" s="6"/>
       <c r="D23" s="7"/>
       <c r="E23" s="8"/>
@@ -833,7 +853,7 @@
     </row>
     <row r="26" spans="1:12" ht="16.5" customHeight="1">
       <c r="A26" s="4"/>
-      <c r="B26" s="14"/>
+      <c r="B26" s="15"/>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
       <c r="E26" s="8"/>
@@ -861,7 +881,7 @@
     </row>
     <row r="28" spans="1:12" ht="16.5" customHeight="1">
       <c r="A28" s="4"/>
-      <c r="B28" s="14"/>
+      <c r="B28" s="15"/>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
       <c r="E28" s="8"/>
@@ -903,7 +923,7 @@
     </row>
     <row r="31" spans="1:12" ht="16.5" customHeight="1">
       <c r="A31" s="4"/>
-      <c r="B31" s="14"/>
+      <c r="B31" s="15"/>
       <c r="C31" s="6"/>
       <c r="D31" s="7"/>
       <c r="E31" s="8"/>
@@ -945,7 +965,7 @@
     </row>
     <row r="34" spans="1:12" ht="16.5" customHeight="1">
       <c r="A34" s="4"/>
-      <c r="B34" s="14"/>
+      <c r="B34" s="15"/>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
@@ -987,7 +1007,7 @@
     </row>
     <row r="37" spans="1:12" ht="16.5" customHeight="1">
       <c r="A37" s="4"/>
-      <c r="B37" s="14"/>
+      <c r="B37" s="15"/>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
       <c r="E37" s="8"/>
@@ -1029,7 +1049,7 @@
     </row>
     <row r="40" spans="1:12" ht="16.5" customHeight="1">
       <c r="A40" s="4"/>
-      <c r="B40" s="14"/>
+      <c r="B40" s="15"/>
       <c r="C40" s="6"/>
       <c r="D40" s="7"/>
       <c r="E40" s="8"/>
@@ -1071,7 +1091,7 @@
     </row>
     <row r="43" spans="1:12" ht="16.5" customHeight="1">
       <c r="A43" s="4"/>
-      <c r="B43" s="14"/>
+      <c r="B43" s="15"/>
       <c r="C43" s="6"/>
       <c r="D43" s="7"/>
       <c r="E43" s="8"/>
@@ -1113,7 +1133,7 @@
     </row>
     <row r="46" spans="1:12" ht="86.25" customHeight="1">
       <c r="A46" s="4"/>
-      <c r="B46" s="14"/>
+      <c r="B46" s="15"/>
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
       <c r="E46" s="8"/>
@@ -1127,10 +1147,10 @@
     </row>
     <row r="47" spans="1:12" ht="16.5" customHeight="1">
       <c r="A47" s="4"/>
-      <c r="B47" s="14"/>
+      <c r="B47" s="15"/>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="15"/>
+      <c r="E47" s="16"/>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
@@ -1155,7 +1175,7 @@
     </row>
     <row r="49" spans="1:12" ht="16.5" customHeight="1">
       <c r="A49" s="4"/>
-      <c r="B49" s="14"/>
+      <c r="B49" s="15"/>
       <c r="C49" s="6"/>
       <c r="D49" s="7"/>
       <c r="E49" s="8"/>
@@ -1169,7 +1189,7 @@
     </row>
     <row r="50" spans="1:12" ht="16.5" customHeight="1">
       <c r="A50" s="4"/>
-      <c r="B50" s="14"/>
+      <c r="B50" s="15"/>
       <c r="C50" s="6"/>
       <c r="D50" s="7"/>
       <c r="E50" s="8"/>
@@ -1211,7 +1231,7 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53" s="4"/>
-      <c r="B53" s="14"/>
+      <c r="B53" s="15"/>
       <c r="C53" s="6"/>
       <c r="D53" s="7"/>
       <c r="E53" s="8"/>

</xml_diff>

<commit_message>
Added slides, deepnote, and prep for 5/6
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,32 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricF\Documents\Teaching\MATH2025FA25\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A283CC8-9CD0-4152-88DB-76DD0E7AD055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <bookViews>
-    <workbookView xWindow="3195" yWindow="2670" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr fullPrecision="1" calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="49" count="66">
   <si>
     <t>Publish</t>
   </si>
@@ -157,7 +145,16 @@
     <t>/prepare/prep-06.qmd</t>
   </si>
   <si>
-    <t>TBD</t>
+    <t>/slides/06-slr-confidence-intervals.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/cofi-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-05-Hypothesis-Testing-Duplicate-Duplicate-f1252cbb-0fe5-4c0d-ada5-1a9c498a6834/%2Fae-06-sbi-ci.qmd?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=f1252cbb-0fe5-4c0d-ada5-1a9c498a6834</t>
+  </si>
+  <si>
+    <t>Mathematical Models for Inference</t>
+  </si>
+  <si>
+    <t>/prepare/prep-07.qmd</t>
   </si>
   <si>
     <t>Homework 2 Due</t>
@@ -169,123 +166,144 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Open Sans"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Open Sans"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="1"/>
       <color rgb="FF334052"/>
       <name val="Inter, sans-serif"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="1"/>
-      <color rgb="FF334052"/>
-      <name val="Inter, sans-serif"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="0"/>
+      <color rgb="FF334052"/>
+      <name val="Inter, sans-serif"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF334052"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <u val="single"/>
       <sz val="11"/>
       <color rgb="FF467886"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFB0280"/>
       <name val="Open Sans"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF334052"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <charset val="0"/>
     </font>
   </fonts>
   <fills count="7">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <fgColor indexed="64"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor indexed="64"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF46BDC6"/>
-        <bgColor rgb="FF339966"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF6D01"/>
-        <bgColor rgb="FFFF9900"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD4D4D4"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -295,474 +313,96 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="16" fontId="6" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="11" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyFill="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Sheet1LockedColumnStyle" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Sheet1LockedColumnStyle" xfId="20"/>
+    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="21"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFB0280"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF006100"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD4D4D4"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF46BDC6"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6D01"/>
-      <rgbColor rgb="FF467886"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF334052"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0"/>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr/>
   <dimension ref="A1:L53"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr customHeight="true" defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="41" customWidth="1"/>
   </cols>
@@ -977,7 +617,7 @@
       <c r="G7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="11" t="s">
         <v>37</v>
       </c>
       <c r="I7" s="9"/>
@@ -1002,7 +642,7 @@
       <c r="F8" s="9"/>
       <c r="G8" s="6"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>40</v>
       </c>
       <c r="J8" s="9"/>
@@ -1028,8 +668,12 @@
       <c r="F9" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+      <c r="G9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>44</v>
+      </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
       <c r="K9" s="4"/>
@@ -1042,16 +686,18 @@
       <c r="B10" s="5">
         <v>7</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="7">
         <v>45924</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="9"/>
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>46</v>
+      </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="9"/>
@@ -1071,13 +717,13 @@
         <v>45925</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="18" t="s">
-        <v>45</v>
+      <c r="I11" s="14" t="s">
+        <v>48</v>
       </c>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
@@ -1177,7 +823,7 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="14"/>
+      <c r="J18" s="15"/>
       <c r="K18" s="6"/>
       <c r="L18" s="9"/>
     </row>
@@ -1225,7 +871,7 @@
     </row>
     <row r="22" spans="1:12" ht="16.5" customHeight="1">
       <c r="A22" s="4"/>
-      <c r="B22" s="15"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="6"/>
       <c r="D22" s="7"/>
       <c r="E22" s="8"/>
@@ -1239,7 +885,7 @@
     </row>
     <row r="23" spans="1:12" ht="16.5" customHeight="1">
       <c r="A23" s="4"/>
-      <c r="B23" s="15"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="6"/>
       <c r="D23" s="7"/>
       <c r="E23" s="8"/>
@@ -1281,7 +927,7 @@
     </row>
     <row r="26" spans="1:12" ht="16.5" customHeight="1">
       <c r="A26" s="4"/>
-      <c r="B26" s="15"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
       <c r="E26" s="8"/>
@@ -1309,7 +955,7 @@
     </row>
     <row r="28" spans="1:12" ht="16.5" customHeight="1">
       <c r="A28" s="4"/>
-      <c r="B28" s="15"/>
+      <c r="B28" s="16"/>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
       <c r="E28" s="8"/>
@@ -1351,7 +997,7 @@
     </row>
     <row r="31" spans="1:12" ht="16.5" customHeight="1">
       <c r="A31" s="4"/>
-      <c r="B31" s="15"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="6"/>
       <c r="D31" s="7"/>
       <c r="E31" s="8"/>
@@ -1393,7 +1039,7 @@
     </row>
     <row r="34" spans="1:12" ht="16.5" customHeight="1">
       <c r="A34" s="4"/>
-      <c r="B34" s="15"/>
+      <c r="B34" s="16"/>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
@@ -1435,7 +1081,7 @@
     </row>
     <row r="37" spans="1:12" ht="16.5" customHeight="1">
       <c r="A37" s="4"/>
-      <c r="B37" s="15"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
       <c r="E37" s="8"/>
@@ -1477,7 +1123,7 @@
     </row>
     <row r="40" spans="1:12" ht="16.5" customHeight="1">
       <c r="A40" s="4"/>
-      <c r="B40" s="15"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="6"/>
       <c r="D40" s="7"/>
       <c r="E40" s="8"/>
@@ -1519,7 +1165,7 @@
     </row>
     <row r="43" spans="1:12" ht="16.5" customHeight="1">
       <c r="A43" s="4"/>
-      <c r="B43" s="15"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="6"/>
       <c r="D43" s="7"/>
       <c r="E43" s="8"/>
@@ -1561,7 +1207,7 @@
     </row>
     <row r="46" spans="1:12" ht="86.25" customHeight="1">
       <c r="A46" s="4"/>
-      <c r="B46" s="15"/>
+      <c r="B46" s="16"/>
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
       <c r="E46" s="8"/>
@@ -1575,10 +1221,10 @@
     </row>
     <row r="47" spans="1:12" ht="16.5" customHeight="1">
       <c r="A47" s="4"/>
-      <c r="B47" s="15"/>
+      <c r="B47" s="16"/>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="16"/>
+      <c r="E47" s="17"/>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
@@ -1603,7 +1249,7 @@
     </row>
     <row r="49" spans="1:12" ht="16.5" customHeight="1">
       <c r="A49" s="4"/>
-      <c r="B49" s="15"/>
+      <c r="B49" s="16"/>
       <c r="C49" s="6"/>
       <c r="D49" s="7"/>
       <c r="E49" s="8"/>
@@ -1617,7 +1263,7 @@
     </row>
     <row r="50" spans="1:12" ht="16.5" customHeight="1">
       <c r="A50" s="4"/>
-      <c r="B50" s="15"/>
+      <c r="B50" s="16"/>
       <c r="C50" s="6"/>
       <c r="D50" s="7"/>
       <c r="E50" s="8"/>
@@ -1657,9 +1303,9 @@
       <c r="K52" s="9"/>
       <c r="L52" s="9"/>
     </row>
-    <row r="53" spans="1:12" ht="16.5">
+    <row r="53" spans="1:12" ht="16.5" customHeight="1">
       <c r="A53" s="4"/>
-      <c r="B53" s="15"/>
+      <c r="B53" s="16"/>
       <c r="C53" s="6"/>
       <c r="D53" s="7"/>
       <c r="E53" s="8"/>
@@ -1672,7 +1318,8 @@
       <c r="L53" s="6"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added prediction and assumptions slides
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,470 +1,415 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr fullPrecision="1" calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="53">
-  <si>
-    <t xml:space="preserve">Publish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lecture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">topic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prepare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">slides</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">project</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eric's Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welcome to MATH 2025!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/00-welcome.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welcome!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Big Picture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/prepare/prep-01.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/01-big-picture.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-01-Getting-Started-f838426f-b7b7-45f4-87a9-5b7c929aa823/notebook/ae-01-getting-started-626fe75c7a02400584058fd9dc0e23ad?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=f838426f-b7b7-45f4-87a9-5b7c929aa823</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Our first AE!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multivariate Relationships</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/prepare/prep-02.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/02-multivariate-relationships.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-02-Multivariate-Relationships-ebce91c8-0f2f-47fd-a6ef-c4d663f9235b/notebook/ae-02-multivariate-relationships-11ff27b42b2c4545b0f393095f59683b?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=ebce91c8-0f2f-47fd-a6ef-c4d663f9235b</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56" count="84">
+  <si>
+    <t>Publish</t>
+  </si>
+  <si>
+    <t>lecture</t>
+  </si>
+  <si>
+    <t>dow</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>topic</t>
+  </si>
+  <si>
+    <t>prepare</t>
+  </si>
+  <si>
+    <t>slides</t>
+  </si>
+  <si>
+    <t>ae</t>
+  </si>
+  <si>
+    <t>hw</t>
+  </si>
+  <si>
+    <t>project</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>Eric's Notes</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Welcome to MATH 2025!</t>
+  </si>
+  <si>
+    <t>/slides/00-welcome.qmd</t>
+  </si>
+  <si>
+    <t>Welcome!</t>
+  </si>
+  <si>
+    <t>The Big Picture</t>
+  </si>
+  <si>
+    <t>/prepare/prep-01.qmd</t>
+  </si>
+  <si>
+    <t>/slides/01-big-picture.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-01-Getting-Started-f838426f-b7b7-45f4-87a9-5b7c929aa823/notebook/ae-01-getting-started-626fe75c7a02400584058fd9dc0e23ad?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=f838426f-b7b7-45f4-87a9-5b7c929aa823</t>
+  </si>
+  <si>
+    <t>Our first AE!</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>Multivariate Relationships</t>
+  </si>
+  <si>
+    <t>/prepare/prep-02.qmd</t>
+  </si>
+  <si>
+    <t>/slides/02-multivariate-relationships.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-02-Multivariate-Relationships-ebce91c8-0f2f-47fd-a6ef-c4d663f9235b/notebook/ae-02-multivariate-relationships-11ff27b42b2c4545b0f393095f59683b?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=ebce91c8-0f2f-47fd-a6ef-c4d663f9235b</t>
   </si>
   <si>
     <t xml:space="preserve">Introduction to Simple Linear Regression </t>
   </si>
   <si>
-    <t xml:space="preserve">/prepare/prep-03.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/03-slr-intro.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-03-Bikeshare-e02ff833-6768-42e4-8b5d-a62f201324b2/Dockerfile?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=e02ff833-6768-42e4-8b5d-a62f201324b2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prediction and Testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/prepare/prep-04.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/04-slr-fit-prediction.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypothesis Testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/prepare/prep-05.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/05-slr-hypothesis-testing.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-05-Hypothesis-Testing-a50d53f1-7c77-4add-8c8b-898d3ea049d6/notebook/ae-05-sbi-ht-82aa13654bfb4659bfce3a86d4d4c28e?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=a50d53f1-7c77-4add-8c8b-898d3ea049d6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homework 1 Due</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/HW-01-e222521f-0b92-4988-9bb5-c8391d9b9270/notebook/hw-01-414692797888442ba6887e84d8f6baca?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=e222521f-0b92-4988-9bb5-c8391d9b9270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypothesis Testing and Intervals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/prepare/prep-06.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidence Intervals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/06-slr-confidence-intervals.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/cofi-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-05-Hypothesis-Testing-Duplicate-Duplicate-f1252cbb-0fe5-4c0d-ada5-1a9c498a6834/%2Fae-06-sbi-ci.qmd?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=f1252cbb-0fe5-4c0d-ada5-1a9c498a6834</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homework 2 Due</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/HW-02-771b407f-d49a-4b32-b1c7-420e5b83e39b/notebook/hw-02-4d1f5e93a5dd43eb875800347e8894c7?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=771b407f-d49a-4b32-b1c7-420e5b83e39b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mathematical Models for Inference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/prepare/prep-08.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/slides/07-slr-math-models.qmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://deepnote.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mathematical Models for Inference (Continued)</t>
+    <t>/prepare/prep-03.qmd</t>
+  </si>
+  <si>
+    <t>/slides/03-slr-intro.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-03-Bikeshare-e02ff833-6768-42e4-8b5d-a62f201324b2/Dockerfile?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=e02ff833-6768-42e4-8b5d-a62f201324b2</t>
+  </si>
+  <si>
+    <t>Prediction and Testing</t>
+  </si>
+  <si>
+    <t>/prepare/prep-04.qmd</t>
+  </si>
+  <si>
+    <t>/slides/04-slr-fit-prediction.qmd</t>
+  </si>
+  <si>
+    <t>Hypothesis Testing</t>
+  </si>
+  <si>
+    <t>/prepare/prep-05.qmd</t>
+  </si>
+  <si>
+    <t>/slides/05-slr-hypothesis-testing.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-05-Hypothesis-Testing-a50d53f1-7c77-4add-8c8b-898d3ea049d6/notebook/ae-05-sbi-ht-82aa13654bfb4659bfce3a86d4d4c28e?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=a50d53f1-7c77-4add-8c8b-898d3ea049d6</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Homework 1 Due</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/HW-01-e222521f-0b92-4988-9bb5-c8391d9b9270/notebook/hw-01-414692797888442ba6887e84d8f6baca?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=e222521f-0b92-4988-9bb5-c8391d9b9270</t>
+  </si>
+  <si>
+    <t>Hypothesis Testing and Intervals</t>
+  </si>
+  <si>
+    <t>/prepare/prep-06.qmd</t>
+  </si>
+  <si>
+    <t>Confidence Intervals</t>
+  </si>
+  <si>
+    <t>/slides/06-slr-confidence-intervals.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/cofi-269748c4-4966-4cc3-b064-2a31b9db85a4/project/AE-05-Hypothesis-Testing-Duplicate-Duplicate-f1252cbb-0fe5-4c0d-ada5-1a9c498a6834/%2Fae-06-sbi-ci.qmd?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=f1252cbb-0fe5-4c0d-ada5-1a9c498a6834</t>
+  </si>
+  <si>
+    <t>Homework 2 Due</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/workspace/CofI-MATH-269748c4-4966-4cc3-b064-2a31b9db85a4/project/HW-02-771b407f-d49a-4b32-b1c7-420e5b83e39b/notebook/hw-02-4d1f5e93a5dd43eb875800347e8894c7?utm_source=share-modal&amp;utm_medium=product-shared-content&amp;utm_campaign=notebook&amp;utm_content=771b407f-d49a-4b32-b1c7-420e5b83e39b</t>
+  </si>
+  <si>
+    <t>Mathematical Models for Inference</t>
+  </si>
+  <si>
+    <t>/prepare/prep-07.qmd</t>
+  </si>
+  <si>
+    <t>/slides/07-slr-math-models.qmd</t>
+  </si>
+  <si>
+    <t>https://deepnote.com/</t>
+  </si>
+  <si>
+    <t>Mathematical Models for Inference (Continued)</t>
+  </si>
+  <si>
+    <t>Prediction and Conditions</t>
+  </si>
+  <si>
+    <t>/prepare/prep-08.qmd</t>
+  </si>
+  <si>
+    <t>/slides/08-slr-prediction.qmd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="d\-mmm"/>
-    <numFmt numFmtId="166" formatCode="h:mm\ AM/PM"/>
-  </numFmts>
-  <fonts count="16">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Aptos Narrow"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Open Sans"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Open Sans"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="1"/>
       <color rgb="FF334052"/>
       <name val="Inter, sans-serif"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="14"/>
       <color rgb="FF334052"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="000563C1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
     </font>
     <font>
       <u val="single"/>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
       <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Open Sans"/>
-      <family val="0"/>
+      <charset val="0"/>
     </font>
     <font>
       <u val="single"/>
       <sz val="11"/>
       <color rgb="FF467886"/>
       <name val="Aptos Narrow"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFB0280"/>
       <name val="Open Sans"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <charset val="0"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <fgColor indexed="64"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor indexed="64"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF46BDC6"/>
-        <bgColor rgb="FF339966"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF6D01"/>
-        <bgColor rgb="FFFF9900"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD4D4D4"/>
-        <bgColor rgb="FFC0C0C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="23">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="42">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="16" fontId="6" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="18" fontId="11" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="22" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="22" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -474,85 +419,25 @@
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Sheet1LockedColumnStyle" xfId="21"/>
-    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="22"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
+    <cellStyle name="Sheet1LockedColumnStyle" xfId="20"/>
+    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="21"/>
+    <cellStyle name="Hyperlink" xfId="22" builtinId="8"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFB0280"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF006100"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0563C1"/>
-      <rgbColor rgb="FFD4D4D4"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF46BDC6"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6D01"/>
-      <rgbColor rgb="FF467886"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF334052"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0"/>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr/>
   <dimension ref="A1:L1048576"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr customHeight="true" defaultRowHeight="14.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="41"/>
+    <col min="7" max="7" width="41" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:12" ht="16.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -590,17 +475,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:12" ht="66" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="5">
         <v>0</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="D2" s="7">
         <v>45896</v>
       </c>
       <c r="E2" s="8" t="s">
@@ -618,23 +503,23 @@
       </c>
       <c r="L2" s="6"/>
     </row>
-    <row r="3" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:12" ht="55.5" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="7">
         <v>45903</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" t="s">
         <v>18</v>
       </c>
       <c r="G3" s="6" t="s">
@@ -650,23 +535,23 @@
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:12" ht="16.5" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="7">
         <v>45908</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="6" t="s">
@@ -680,23 +565,23 @@
       <c r="K4" s="9"/>
       <c r="L4" s="6"/>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:12" ht="16.5" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="5">
         <v>3</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="7">
         <v>45910</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" t="s">
         <v>28</v>
       </c>
       <c r="G5" s="6" t="s">
@@ -710,23 +595,23 @@
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:12" ht="16.5" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="7">
         <v>45915</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" t="s">
         <v>32</v>
       </c>
       <c r="G6" s="6" t="s">
@@ -740,23 +625,23 @@
       <c r="K6" s="9"/>
       <c r="L6" s="6"/>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:12" ht="16.5" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="5">
         <v>5</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="7">
         <v>45917</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" t="s">
         <v>35</v>
       </c>
       <c r="G7" s="6" t="s">
@@ -770,7 +655,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:12" ht="16.5" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
@@ -778,7 +663,7 @@
       <c r="C8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="7">
         <v>45919</v>
       </c>
       <c r="E8" s="8" t="s">
@@ -794,23 +679,23 @@
       <c r="K8" s="9"/>
       <c r="L8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:12" ht="16.5" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="5">
         <v>6</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="7">
         <v>45922</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" t="s">
         <v>42</v>
       </c>
       <c r="G9" s="6" t="s">
@@ -824,29 +709,29 @@
       <c r="K9" s="4"/>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:12" ht="16.5" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="5">
         <v>7</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="7">
         <v>45924</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" t="s">
         <v>42</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="11" t="s">
         <v>45</v>
       </c>
       <c r="I10" s="9"/>
@@ -854,7 +739,7 @@
       <c r="K10" s="4"/>
       <c r="L10" s="9"/>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:12" ht="16.5" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
@@ -862,7 +747,7 @@
       <c r="C11" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="7">
         <v>45925</v>
       </c>
       <c r="E11" s="8" t="s">
@@ -871,30 +756,30 @@
       <c r="F11" s="9"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="13" t="s">
         <v>47</v>
       </c>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
       <c r="L11" s="9"/>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:12" ht="16.5" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="5">
         <v>8</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="7">
         <v>45929</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" t="s">
         <v>49</v>
       </c>
       <c r="G12" s="6" t="s">
@@ -908,24 +793,24 @@
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:12" ht="16.5" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="5">
         <v>9</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="7">
         <v>45931</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>52</v>
       </c>
       <c r="F13" s="9"/>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="6" t="s">
         <v>50</v>
       </c>
       <c r="H13" s="6"/>
@@ -934,21 +819,37 @@
       <c r="K13" s="6"/>
       <c r="L13" s="9"/>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+    <row r="14" spans="1:12" ht="16.5" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="5">
+        <v>10</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="7">
+        <v>45936</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="I14" s="4"/>
       <c r="J14" s="9"/>
       <c r="K14" s="6"/>
       <c r="L14" s="9"/>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:12" ht="16.5" customHeight="1">
       <c r="A15" s="4"/>
       <c r="B15" s="5"/>
       <c r="C15" s="6"/>
@@ -962,7 +863,7 @@
       <c r="K15" s="6"/>
       <c r="L15" s="9"/>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:12" ht="16.5" customHeight="1">
       <c r="A16" s="4"/>
       <c r="B16" s="5"/>
       <c r="C16" s="6"/>
@@ -976,7 +877,7 @@
       <c r="K16" s="6"/>
       <c r="L16" s="9"/>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:12" ht="16.5" customHeight="1">
       <c r="A17" s="4"/>
       <c r="B17" s="5"/>
       <c r="C17" s="6"/>
@@ -990,7 +891,7 @@
       <c r="K17" s="6"/>
       <c r="L17" s="9"/>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:12" ht="16.5" customHeight="1">
       <c r="A18" s="4"/>
       <c r="B18" s="5"/>
       <c r="C18" s="6"/>
@@ -1000,11 +901,11 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="17"/>
+      <c r="J18" s="16"/>
       <c r="K18" s="6"/>
       <c r="L18" s="9"/>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:12" ht="16.5" customHeight="1">
       <c r="A19" s="4"/>
       <c r="B19" s="5"/>
       <c r="C19" s="6"/>
@@ -1018,7 +919,7 @@
       <c r="K19" s="6"/>
       <c r="L19" s="9"/>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:12" ht="16.5" customHeight="1">
       <c r="A20" s="4"/>
       <c r="B20" s="5"/>
       <c r="C20" s="6"/>
@@ -1032,7 +933,7 @@
       <c r="K20" s="9"/>
       <c r="L20" s="9"/>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:12" ht="16.5" customHeight="1">
       <c r="A21" s="4"/>
       <c r="B21" s="5"/>
       <c r="C21" s="6"/>
@@ -1046,9 +947,9 @@
       <c r="K21" s="4"/>
       <c r="L21" s="9"/>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:12" ht="16.5" customHeight="1">
       <c r="A22" s="4"/>
-      <c r="B22" s="18"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="6"/>
       <c r="D22" s="7"/>
       <c r="E22" s="8"/>
@@ -1060,9 +961,9 @@
       <c r="K22" s="9"/>
       <c r="L22" s="9"/>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:12" ht="16.5" customHeight="1">
       <c r="A23" s="4"/>
-      <c r="B23" s="18"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="6"/>
       <c r="D23" s="7"/>
       <c r="E23" s="8"/>
@@ -1074,7 +975,7 @@
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:12" ht="16.5" customHeight="1">
       <c r="A24" s="4"/>
       <c r="B24" s="5"/>
       <c r="C24" s="6"/>
@@ -1088,7 +989,7 @@
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:12" ht="16.5" customHeight="1">
       <c r="A25" s="4"/>
       <c r="B25" s="5"/>
       <c r="C25" s="6"/>
@@ -1102,9 +1003,9 @@
       <c r="K25" s="6"/>
       <c r="L25" s="9"/>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:12" ht="16.5" customHeight="1">
       <c r="A26" s="4"/>
-      <c r="B26" s="18"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
       <c r="E26" s="8"/>
@@ -1116,7 +1017,7 @@
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
     </row>
-    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:12" ht="16.5" customHeight="1">
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
@@ -1130,9 +1031,9 @@
       <c r="K27" s="9"/>
       <c r="L27" s="9"/>
     </row>
-    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:12" ht="16.5" customHeight="1">
       <c r="A28" s="4"/>
-      <c r="B28" s="18"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
       <c r="E28" s="8"/>
@@ -1144,7 +1045,7 @@
       <c r="K28" s="9"/>
       <c r="L28" s="9"/>
     </row>
-    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:12" ht="16.5" customHeight="1">
       <c r="A29" s="4"/>
       <c r="B29" s="5"/>
       <c r="C29" s="6"/>
@@ -1158,7 +1059,7 @@
       <c r="K29" s="9"/>
       <c r="L29" s="9"/>
     </row>
-    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:12" ht="16.5" customHeight="1">
       <c r="A30" s="4"/>
       <c r="B30" s="5"/>
       <c r="C30" s="6"/>
@@ -1172,9 +1073,9 @@
       <c r="K30" s="9"/>
       <c r="L30" s="9"/>
     </row>
-    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:12" ht="16.5" customHeight="1">
       <c r="A31" s="4"/>
-      <c r="B31" s="18"/>
+      <c r="B31" s="17"/>
       <c r="C31" s="6"/>
       <c r="D31" s="7"/>
       <c r="E31" s="8"/>
@@ -1186,7 +1087,7 @@
       <c r="K31" s="9"/>
       <c r="L31" s="6"/>
     </row>
-    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:12" ht="16.5" customHeight="1">
       <c r="A32" s="4"/>
       <c r="B32" s="5"/>
       <c r="C32" s="6"/>
@@ -1200,7 +1101,7 @@
       <c r="K32" s="9"/>
       <c r="L32" s="9"/>
     </row>
-    <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:12" ht="16.5" customHeight="1">
       <c r="A33" s="4"/>
       <c r="B33" s="5"/>
       <c r="C33" s="6"/>
@@ -1214,9 +1115,9 @@
       <c r="K33" s="9"/>
       <c r="L33" s="9"/>
     </row>
-    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:12" ht="16.5" customHeight="1">
       <c r="A34" s="4"/>
-      <c r="B34" s="18"/>
+      <c r="B34" s="17"/>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
@@ -1228,7 +1129,7 @@
       <c r="K34" s="9"/>
       <c r="L34" s="9"/>
     </row>
-    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:12" ht="16.5" customHeight="1">
       <c r="A35" s="4"/>
       <c r="B35" s="5"/>
       <c r="C35" s="6"/>
@@ -1242,7 +1143,7 @@
       <c r="K35" s="9"/>
       <c r="L35" s="9"/>
     </row>
-    <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:12" ht="16.5" customHeight="1">
       <c r="A36" s="4"/>
       <c r="B36" s="5"/>
       <c r="C36" s="6"/>
@@ -1256,9 +1157,9 @@
       <c r="K36" s="6"/>
       <c r="L36" s="9"/>
     </row>
-    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:12" ht="16.5" customHeight="1">
       <c r="A37" s="4"/>
-      <c r="B37" s="18"/>
+      <c r="B37" s="17"/>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
       <c r="E37" s="8"/>
@@ -1270,7 +1171,7 @@
       <c r="K37" s="9"/>
       <c r="L37" s="9"/>
     </row>
-    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:12" ht="16.5" customHeight="1">
       <c r="A38" s="4"/>
       <c r="B38" s="5"/>
       <c r="C38" s="6"/>
@@ -1284,7 +1185,7 @@
       <c r="K38" s="9"/>
       <c r="L38" s="9"/>
     </row>
-    <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:12" ht="16.5" customHeight="1">
       <c r="A39" s="4"/>
       <c r="B39" s="5"/>
       <c r="C39" s="6"/>
@@ -1298,9 +1199,9 @@
       <c r="K39" s="6"/>
       <c r="L39" s="9"/>
     </row>
-    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:12" ht="16.5" customHeight="1">
       <c r="A40" s="4"/>
-      <c r="B40" s="18"/>
+      <c r="B40" s="17"/>
       <c r="C40" s="6"/>
       <c r="D40" s="7"/>
       <c r="E40" s="8"/>
@@ -1312,7 +1213,7 @@
       <c r="K40" s="9"/>
       <c r="L40" s="9"/>
     </row>
-    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:12" ht="16.5" customHeight="1">
       <c r="A41" s="4"/>
       <c r="B41" s="5"/>
       <c r="C41" s="6"/>
@@ -1326,7 +1227,7 @@
       <c r="K41" s="9"/>
       <c r="L41" s="9"/>
     </row>
-    <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:12" ht="16.5" customHeight="1">
       <c r="A42" s="4"/>
       <c r="B42" s="5"/>
       <c r="C42" s="6"/>
@@ -1340,9 +1241,9 @@
       <c r="K42" s="6"/>
       <c r="L42" s="9"/>
     </row>
-    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:12" ht="16.5" customHeight="1">
       <c r="A43" s="4"/>
-      <c r="B43" s="18"/>
+      <c r="B43" s="17"/>
       <c r="C43" s="6"/>
       <c r="D43" s="7"/>
       <c r="E43" s="8"/>
@@ -1354,7 +1255,7 @@
       <c r="K43" s="9"/>
       <c r="L43" s="6"/>
     </row>
-    <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:12" ht="16.5" customHeight="1">
       <c r="A44" s="4"/>
       <c r="B44" s="5"/>
       <c r="C44" s="6"/>
@@ -1368,7 +1269,7 @@
       <c r="K44" s="9"/>
       <c r="L44" s="9"/>
     </row>
-    <row r="45" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:12" ht="16.5" customHeight="1">
       <c r="A45" s="4"/>
       <c r="B45" s="5"/>
       <c r="C45" s="6"/>
@@ -1382,9 +1283,9 @@
       <c r="K45" s="6"/>
       <c r="L45" s="9"/>
     </row>
-    <row r="46" customFormat="false" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:12" ht="86.25" customHeight="1">
       <c r="A46" s="4"/>
-      <c r="B46" s="18"/>
+      <c r="B46" s="17"/>
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
       <c r="E46" s="8"/>
@@ -1396,12 +1297,12 @@
       <c r="K46" s="9"/>
       <c r="L46" s="6"/>
     </row>
-    <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:12" ht="16.5" customHeight="1">
       <c r="A47" s="4"/>
-      <c r="B47" s="18"/>
+      <c r="B47" s="17"/>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="19"/>
+      <c r="E47" s="18"/>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
@@ -1410,7 +1311,7 @@
       <c r="K47" s="9"/>
       <c r="L47" s="9"/>
     </row>
-    <row r="48" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:12" ht="16.5" customHeight="1">
       <c r="A48" s="4"/>
       <c r="B48" s="5"/>
       <c r="C48" s="6"/>
@@ -1424,9 +1325,9 @@
       <c r="K48" s="9"/>
       <c r="L48" s="6"/>
     </row>
-    <row r="49" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:12" ht="16.5" customHeight="1">
       <c r="A49" s="4"/>
-      <c r="B49" s="18"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="6"/>
       <c r="D49" s="7"/>
       <c r="E49" s="8"/>
@@ -1438,9 +1339,9 @@
       <c r="K49" s="6"/>
       <c r="L49" s="9"/>
     </row>
-    <row r="50" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:12" ht="16.5" customHeight="1">
       <c r="A50" s="4"/>
-      <c r="B50" s="18"/>
+      <c r="B50" s="17"/>
       <c r="C50" s="6"/>
       <c r="D50" s="7"/>
       <c r="E50" s="8"/>
@@ -1452,7 +1353,7 @@
       <c r="K50" s="9"/>
       <c r="L50" s="9"/>
     </row>
-    <row r="51" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:12" ht="16.5" customHeight="1">
       <c r="A51" s="4"/>
       <c r="B51" s="5"/>
       <c r="C51" s="6"/>
@@ -1466,7 +1367,7 @@
       <c r="K51" s="9"/>
       <c r="L51" s="9"/>
     </row>
-    <row r="52" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:12" ht="16.5" customHeight="1">
       <c r="A52" s="4"/>
       <c r="B52" s="5"/>
       <c r="C52" s="6"/>
@@ -1480,9 +1381,9 @@
       <c r="K52" s="9"/>
       <c r="L52" s="9"/>
     </row>
-    <row r="53" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:12" ht="16.5" customHeight="1">
       <c r="A53" s="4"/>
-      <c r="B53" s="18"/>
+      <c r="B53" s="17"/>
       <c r="C53" s="6"/>
       <c r="D53" s="7"/>
       <c r="E53" s="8"/>
@@ -1494,17 +1395,14 @@
       <c r="K53" s="9"/>
       <c r="L53" s="6"/>
     </row>
-    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" ht="12.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H12" r:id="rId1" display="https://deepnote.com/"/>
+    <hyperlink ref="H14" r:id="rId2" display="https://deepnote.com/"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Exam to Schedule
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="59" count="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="60" count="98">
   <si>
     <t>Publish</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t>/ae/ae-09-exam01-handwritten.qmd</t>
+  </si>
+  <si>
+    <t>Exam 1</t>
   </si>
 </sst>
 </file>
@@ -917,11 +920,21 @@
       <c r="L16" s="9"/>
     </row>
     <row r="17" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="8"/>
+      <c r="A17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5">
+        <v>13</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="7">
+        <v>45945</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>59</v>
+      </c>
       <c r="F17" s="9"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>

</xml_diff>

<commit_message>
Added next lecture hw and activities
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="60" count="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="63" count="106">
   <si>
     <t>Publish</t>
   </si>
@@ -194,6 +194,15 @@
   </si>
   <si>
     <t>Exam 1</t>
+  </si>
+  <si>
+    <t>Model Evaluation and ANOVA</t>
+  </si>
+  <si>
+    <t>/slides/10-model-eval.qmd</t>
+  </si>
+  <si>
+    <t>Transformations and Outliers</t>
   </si>
 </sst>
 </file>
@@ -447,6 +456,7 @@
   <sheetFormatPr customHeight="true" defaultRowHeight="14.25"/>
   <cols>
     <col min="7" max="7" width="41" customWidth="1"/>
+    <col min="8" max="8" width="255" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="16.5" customHeight="1">
@@ -944,25 +954,49 @@
       <c r="L17" s="9"/>
     </row>
     <row r="18" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A18" s="4"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="8"/>
+      <c r="A18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="5">
+        <v>14</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="7">
+        <v>45950</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="F18" s="9"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
+      <c r="G18" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="I18" s="8"/>
       <c r="J18" s="16"/>
       <c r="K18" s="6"/>
       <c r="L18" s="9"/>
     </row>
     <row r="19" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="8"/>
+      <c r="A19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="5">
+        <v>15</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="7">
+        <v>45952</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1453,6 +1487,7 @@
     <hyperlink ref="H12" r:id="rId1" display="https://deepnote.com/"/>
     <hyperlink ref="H14" r:id="rId2" display="https://deepnote.com/"/>
     <hyperlink ref="H15" r:id="rId3" display="https://deepnote.com/"/>
+    <hyperlink ref="H18" r:id="rId4" display="https://deepnote.com/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>

</xml_diff>

<commit_message>
Added slides for 16
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricF\Documents\Teaching\MATH2025FA25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85EC10C-8F85-4C07-9F68-289E317A8C73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B062EC89-4A58-4E92-8499-2C9150D81243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="76">
   <si>
     <t>Publish</t>
   </si>
@@ -242,6 +242,12 @@
   </si>
   <si>
     <t>/slides/15-mlr-inference.qmd</t>
+  </si>
+  <si>
+    <t>MLR: Conditions</t>
+  </si>
+  <si>
+    <t>/slides/16-mlr-conditions.qmd</t>
   </si>
 </sst>
 </file>
@@ -1400,14 +1406,28 @@
       <c r="L23" s="9"/>
     </row>
     <row r="24" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A24" s="4"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="8"/>
+      <c r="A24" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="5">
+        <v>20</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="7">
+        <v>45971</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>74</v>
+      </c>
       <c r="F24" s="9"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="9"/>
+      <c r="G24" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>51</v>
+      </c>
       <c r="I24" s="6"/>
       <c r="J24" s="9"/>
       <c r="K24" s="9"/>
@@ -1831,6 +1851,7 @@
     <hyperlink ref="H21" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="H22" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="H23" r:id="rId9" xr:uid="{4739ECB5-1331-49F7-B13E-B6B1E046166A}"/>
+    <hyperlink ref="H24" r:id="rId10" xr:uid="{C759B772-F64A-4719-A029-E975DB3867DC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>

<commit_message>
Added MC lecture and updated schedule
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricF\Documents\Teaching\MATH2025FA25\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B062EC89-4A58-4E92-8499-2C9150D81243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr fullPrecision="1" calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="85" count="166">
   <si>
     <t>Publish</t>
   </si>
@@ -235,102 +229,170 @@
     <t>/slides/14-categorical-predictors.qmd</t>
   </si>
   <si>
+    <t>MLR: Inference</t>
+  </si>
+  <si>
+    <t>/slides/15-mlr-inference.qmd</t>
+  </si>
+  <si>
     <t>/project/project-pilot.qmd</t>
   </si>
   <si>
-    <t>MLR: Inference</t>
-  </si>
-  <si>
-    <t>/slides/15-mlr-inference.qmd</t>
-  </si>
-  <si>
     <t>MLR: Conditions</t>
   </si>
   <si>
     <t>/slides/16-mlr-conditions.qmd</t>
+  </si>
+  <si>
+    <t>MLR Conditions Cont.</t>
+  </si>
+  <si>
+    <t>Multicollinearity</t>
+  </si>
+  <si>
+    <t>/slides/17-multicollinearity.qmd</t>
+  </si>
+  <si>
+    <t>Model Selection</t>
+  </si>
+  <si>
+    <t>No Class Thanksgiving Break</t>
+  </si>
+  <si>
+    <t>Final Exam Review</t>
+  </si>
+  <si>
+    <t>Final Exam</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Poster Session</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Aptos Narrow"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Open Sans"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Open Sans"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="1"/>
       <color rgb="FF334052"/>
       <name val="Inter, sans-serif"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <charset val="0"/>
     </font>
     <font>
       <sz val="14"/>
       <color rgb="FF334052"/>
       <name val="Arial"/>
+      <charset val="0"/>
     </font>
     <font>
-      <u/>
+      <u val="single"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="000563C1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <u val="single"/>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
       <name val="Calibri"/>
+      <charset val="0"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
+      <u val="single"/>
       <sz val="11"/>
       <color rgb="FF467886"/>
       <name val="Aptos Narrow"/>
+      <charset val="0"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFB0280"/>
       <name val="Open Sans"/>
+      <charset val="0"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <fgColor indexed="64"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor indexed="64"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -381,360 +443,83 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="16" fontId="6" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="11" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="22" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="22" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyBorder="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
+  <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Sheet1LockedColumnStyle" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Sheet1LockedColumnStyle" xfId="20"/>
+    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="21"/>
+    <cellStyle name="Hyperlink" xfId="22" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="44546A"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4472C4"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="ED7D31"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="FFC000"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="70AD47"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0563C1"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="954F72"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
-      <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr/>
   <dimension ref="A1:L1048576"/>
-  <sheetFormatPr defaultRowHeight="14.25" customHeight="1"/>
+  <sheetFormatPr customHeight="true" defaultRowHeight="14.25"/>
   <cols>
     <col min="7" max="7" width="41" customWidth="1"/>
     <col min="8" max="8" width="255" customWidth="1"/>
@@ -1088,7 +873,7 @@
       <c r="G12" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H12" s="14" t="s">
+      <c r="H12" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I12" s="9"/>
@@ -1144,7 +929,7 @@
       <c r="G14" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I14" s="4"/>
@@ -1174,7 +959,7 @@
       <c r="G15" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I15" s="9"/>
@@ -1254,11 +1039,11 @@
       <c r="G18" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="H18" s="14" t="s">
+      <c r="H18" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I18" s="8"/>
-      <c r="J18" s="15"/>
+      <c r="J18" s="16"/>
       <c r="K18" s="6"/>
       <c r="L18" s="9"/>
     </row>
@@ -1282,7 +1067,7 @@
       <c r="G19" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="14" t="s">
+      <c r="H19" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I19" s="8"/>
@@ -1310,7 +1095,7 @@
       <c r="G20" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H20" s="14" t="s">
+      <c r="H20" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I20" s="8"/>
@@ -1338,7 +1123,7 @@
       <c r="G21" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="H21" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I21" s="9"/>
@@ -1368,7 +1153,7 @@
       <c r="G22" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="H22" s="14" t="s">
+      <c r="H22" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I22" s="9"/>
@@ -1389,18 +1174,18 @@
         <v>45966</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="H23" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
@@ -1425,7 +1210,7 @@
       <c r="G24" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="H24" s="14" t="s">
+      <c r="H24" s="15" t="s">
         <v>51</v>
       </c>
       <c r="I24" s="6"/>
@@ -1434,39 +1219,77 @@
       <c r="L24" s="9"/>
     </row>
     <row r="25" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A25" s="4"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="8"/>
+      <c r="A25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="5">
+        <v>21</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="7">
+        <v>45973</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="F25" s="9"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="9"/>
+      <c r="G25" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="I25" s="6"/>
       <c r="J25" s="9"/>
       <c r="K25" s="6"/>
       <c r="L25" s="9"/>
     </row>
     <row r="26" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A26" s="4"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="8"/>
+      <c r="A26" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="5">
+        <v>22</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D26" s="7">
+        <v>45978</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>77</v>
+      </c>
       <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
+      <c r="G26" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="I26" s="9"/>
       <c r="J26" s="9"/>
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
     </row>
     <row r="27" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A27" s="4"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="8"/>
+      <c r="A27" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" s="5">
+        <v>23</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="7">
+        <v>45980</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>79</v>
+      </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
@@ -1476,11 +1299,21 @@
       <c r="L27" s="9"/>
     </row>
     <row r="28" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A28" s="4"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="7">
+        <v>45985</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
       <c r="H28" s="9"/>
@@ -1490,11 +1323,21 @@
       <c r="L28" s="9"/>
     </row>
     <row r="29" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A29" s="4"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="8"/>
+      <c r="A29" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="7">
+        <v>45987</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -1504,11 +1347,21 @@
       <c r="L29" s="9"/>
     </row>
     <row r="30" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A30" s="4"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="8"/>
+      <c r="A30" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="5">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D30" s="7">
+        <v>45992</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
@@ -1518,11 +1371,21 @@
       <c r="L30" s="9"/>
     </row>
     <row r="31" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A31" s="4"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="8"/>
+      <c r="A31" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="5">
+        <v>25</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="7">
+        <v>45994</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>82</v>
+      </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
@@ -1532,11 +1395,21 @@
       <c r="L31" s="6"/>
     </row>
     <row r="32" spans="1:12" ht="16.5" customHeight="1">
-      <c r="A32" s="4"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="8"/>
+      <c r="A32" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="7">
+        <v>46001</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>84</v>
+      </c>
       <c r="F32" s="9"/>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
@@ -1561,7 +1434,7 @@
     </row>
     <row r="34" spans="1:12" ht="16.5" customHeight="1">
       <c r="A34" s="4"/>
-      <c r="B34" s="16"/>
+      <c r="B34" s="17"/>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
       <c r="E34" s="8"/>
@@ -1603,7 +1476,7 @@
     </row>
     <row r="37" spans="1:12" ht="16.5" customHeight="1">
       <c r="A37" s="4"/>
-      <c r="B37" s="16"/>
+      <c r="B37" s="17"/>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
       <c r="E37" s="8"/>
@@ -1645,7 +1518,7 @@
     </row>
     <row r="40" spans="1:12" ht="16.5" customHeight="1">
       <c r="A40" s="4"/>
-      <c r="B40" s="16"/>
+      <c r="B40" s="17"/>
       <c r="C40" s="6"/>
       <c r="D40" s="7"/>
       <c r="E40" s="8"/>
@@ -1687,7 +1560,7 @@
     </row>
     <row r="43" spans="1:12" ht="16.5" customHeight="1">
       <c r="A43" s="4"/>
-      <c r="B43" s="16"/>
+      <c r="B43" s="17"/>
       <c r="C43" s="6"/>
       <c r="D43" s="7"/>
       <c r="E43" s="8"/>
@@ -1729,7 +1602,7 @@
     </row>
     <row r="46" spans="1:12" ht="86.25" customHeight="1">
       <c r="A46" s="4"/>
-      <c r="B46" s="16"/>
+      <c r="B46" s="17"/>
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
       <c r="E46" s="8"/>
@@ -1743,10 +1616,10 @@
     </row>
     <row r="47" spans="1:12" ht="16.5" customHeight="1">
       <c r="A47" s="4"/>
-      <c r="B47" s="16"/>
+      <c r="B47" s="17"/>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="17"/>
+      <c r="E47" s="18"/>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
@@ -1771,7 +1644,7 @@
     </row>
     <row r="49" spans="1:12" ht="16.5" customHeight="1">
       <c r="A49" s="4"/>
-      <c r="B49" s="16"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="6"/>
       <c r="D49" s="7"/>
       <c r="E49" s="8"/>
@@ -1785,7 +1658,7 @@
     </row>
     <row r="50" spans="1:12" ht="16.5" customHeight="1">
       <c r="A50" s="4"/>
-      <c r="B50" s="16"/>
+      <c r="B50" s="17"/>
       <c r="C50" s="6"/>
       <c r="D50" s="7"/>
       <c r="E50" s="8"/>
@@ -1827,7 +1700,7 @@
     </row>
     <row r="53" spans="1:12" ht="16.5" customHeight="1">
       <c r="A53" s="4"/>
-      <c r="B53" s="16"/>
+      <c r="B53" s="17"/>
       <c r="C53" s="6"/>
       <c r="D53" s="7"/>
       <c r="E53" s="8"/>
@@ -1842,18 +1715,21 @@
     <row r="1048576" ht="12.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H12" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="H14" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="H15" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="H18" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="H19" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="H20" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="H21" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="H22" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="H23" r:id="rId9" xr:uid="{4739ECB5-1331-49F7-B13E-B6B1E046166A}"/>
-    <hyperlink ref="H24" r:id="rId10" xr:uid="{C759B772-F64A-4719-A029-E975DB3867DC}"/>
+    <hyperlink ref="H12" r:id="rId1" display="https://deepnote.com/"/>
+    <hyperlink ref="H14" r:id="rId2" display="https://deepnote.com/"/>
+    <hyperlink ref="H15" r:id="rId3" display="https://deepnote.com/"/>
+    <hyperlink ref="H18" r:id="rId4" display="https://deepnote.com/"/>
+    <hyperlink ref="H19" r:id="rId5" display="https://deepnote.com/"/>
+    <hyperlink ref="H20" r:id="rId6" display="https://deepnote.com/"/>
+    <hyperlink ref="H21" r:id="rId7" display="https://deepnote.com/"/>
+    <hyperlink ref="H22" r:id="rId8" display="https://deepnote.com/"/>
+    <hyperlink ref="H23" r:id="rId9" display="https://deepnote.com/"/>
+    <hyperlink ref="H24" r:id="rId10" display="https://deepnote.com/"/>
+    <hyperlink ref="H25" r:id="rId11" display="https://deepnote.com/"/>
+    <hyperlink ref="H26" r:id="rId12" display="https://deepnote.com/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter alignWithMargins="0"/>
+  <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding exam 2 stuff
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EricF\Documents\Teaching\MATH2025FA25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219BB176-C072-407C-8289-0733BBB0248C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F594B723-599D-43E4-8D33-A10845F54CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="88">
   <si>
     <t>Publish</t>
   </si>
@@ -278,6 +278,12 @@
   </si>
   <si>
     <t>/slides/18-comparison.qmd</t>
+  </si>
+  <si>
+    <t>/slides/19-exam-02-review.qmd</t>
+  </si>
+  <si>
+    <t>/ae/ae-19-exam2-practice.qmd</t>
   </si>
 </sst>
 </file>
@@ -1612,8 +1618,12 @@
         <v>80</v>
       </c>
       <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
+      <c r="G30" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>87</v>
+      </c>
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
       <c r="K30" s="9"/>

</xml_diff>